<commit_message>
implemented temporal and spatial augmentation
</commit_message>
<xml_diff>
--- a/Excel Results/results_single.xlsx
+++ b/Excel Results/results_single.xlsx
@@ -1,54 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\hazard_prediction_project\Excel Results\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E32EED-E586-49AE-BEA2-C9C6F5E7FBDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
-  <si>
-    <t>Parameters</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
       <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -78,25 +71,85 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -384,13 +437,953 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C78"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Parameters</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>single_img_input_25</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>single_img_input_25</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>single_img_input</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>single_img_input</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>img_local_context_ROI_1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>img_local_context_ROI_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>7091</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>7091</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>7011</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>7011</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>./output/dataset_cache</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>./output/dataset_cache</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>7011</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>7011</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>CNN_LSTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>literature_classes</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>literature_classes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>0.0002</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>0.0002</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>2e-05</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>2e-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>1e-05</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>1e-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>0.00018</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>0.00018</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLRWarmUp</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>CosineAnnealingLRWarmUp</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>5e-07</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>5e-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>FocalLoss</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>FocalLoss</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>single_img_input_25</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>single_img_input_25</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>0.783</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>0.781</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>0.816</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>0.816</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>0.816</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>0.818</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>0.816</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>0.816</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>0.811</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>0.811</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>0.809</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>0.808</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>0.771</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>0.771</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>